<commit_message>
Fix corrupted files from earlier transfer (batch 17, final)
Re-downloaded 5 files that had silent content corruption despite
matching byte sizes (2 xlsx with bad zip CRC, 2 py with encoding/
syntax corruption); also picked up build_probe.py from the
generators completion pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1.xlsx
@@ -530,4 +530,446 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.2" customWidth="1" min="1" max="1"/>
+    <col width="4.5" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="2.2" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>TRANSFORMER  SPECIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L6790A single-stage PF LLC converter      25 V / 26.3 A output      —      turns ratio 7.5 : 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="4" customHeight="1">
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>1.    CONFIGURATION</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>•   Three identical transformers per set — primaries in series, secondaries in parallel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>•   EVERY VALUE BELOW IS PER TRANSFORMER.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="19" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2.    WINDING</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Winding</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Turns</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Winding current           rms   /   peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>NP1     Primary</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>5 Ts</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>10.9 A   /   18.3 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>NS2     Secondary A</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>3 – 5</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>2 T</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>9.4 A   /   32.9 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>NS3     Secondary B</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>2 T</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>9.4 A   /   32.9 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>NAUX   Auxiliary (ZCD)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>a – b</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>1 T</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>sense only</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Centre tap is made on the PCB by joining pins 4 and 5 — do NOT join them inside the transformer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>3.    ELECTRICAL  REQUIREMENTS</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Measured with an LCR meter at 100 kHz / 1 V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>INDUCTANCE</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>10.33 µH    ±10 %</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>All other windings OPEN.   L.mag + L.leak, not L.mag alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>LEAKAGE INDUCTANCE</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>3.67 µH    ±10 %</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>SECONDARY ALL SHORT (NS2 + NS3).   NAUX open.   Resonant inductor — a target, not a maximum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>D.C OVERLAP</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>≥ 90 % of initial inductance</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Test current 15 A, normal temperature</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14" customHeight="1">
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Both measured at 1 – 2 of ONE transformer.   Three in series give a total ratio of 7.5 : 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="14" customHeight="1">
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Item 2 follows the existing production part 26OP-LM83W clause 4-2, "SECONDARY ALL SHORT" — same vendor, same centre-tapped construction.   The auxiliary is NOT shorted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>4.    OPERATING  CONDITIONS</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Switching frequency</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>92  to  249 kHz</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>at full load</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Core effective area</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Ae  ≥  103 mm²</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>holds the peak flux density at or below 0.20 T</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="14" customHeight="1">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Core, bobbin, wire and winding arrangement are the supplier’s choice, provided section 3 is met.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B17:F17"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Three-core spec: terminals back to the 26OP-LM83W approval-sheet naming (1-2 / 3-5 / 4-6 / a-b, tap at 4-5), no coil former named — the PQ 40/40 pin numbers had crept in from the AN pin figure on 2026-09-22 and were never asked for
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F46"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.2" customWidth="1" min="1" max="1"/>
@@ -553,6 +553,7 @@
     <col width="2.2" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -574,16 +575,13 @@
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6" ht="19" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>1.    CONFIGURATION</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
@@ -599,16 +597,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="19" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>2.    WINDING</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="8" t="inlineStr">
@@ -650,7 +645,7 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>1 – 3</t>
+          <t>1 – 2</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -677,7 +672,7 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>7 – 9</t>
+          <t>3 – 5</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -704,7 +699,7 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>10 – 12</t>
+          <t>4 – 6</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -731,7 +726,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>4 – 6</t>
+          <t>a – b</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -745,17 +740,18 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="14" customHeight="1">
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Centre tap is made on the PCB by joining pins 9 and 10 — do NOT join them inside the transformer.</t>
+          <t>Centre tap is made on the PCB by joining pins 4 and 5 — do NOT join them inside the transformer.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Coil former TDK B65884E (PQ 40/40), 12 pins.   Pin numbers count along one row from pin 1 and back along the other — confirm on the bobbin drawing before winding.</t>
+          <t>Terminal numbers follow the existing production part 26OP-LM83W (approval sheet, KH Feelux): primary 1 – 2, secondaries 3 – 5 and 4 – 6, auxiliary a – b. Core, bobbin and pin layout are the supplier’s choice.</t>
         </is>
       </c>
     </row>
@@ -765,10 +761,6 @@
           <t>3.    ELECTRICAL  REQUIREMENTS</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
     </row>
     <row r="20" ht="14" customHeight="1">
       <c r="B20" s="12" t="inlineStr">
@@ -817,7 +809,7 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>1 – 3</t>
+          <t>1 – 2</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -844,7 +836,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>1 – 3</t>
+          <t>1 – 2</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -871,7 +863,7 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>1 – 3</t>
+          <t>1 – 2</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -888,7 +880,7 @@
     <row r="25" ht="14" customHeight="1">
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Both measured at 1 – 3 of ONE transformer.   Three in series give a total ratio of 7.5 : 1.</t>
+          <t>Both measured at 1 – 2 of ONE transformer.   Three in series give a total ratio of 7.5 : 1.</t>
         </is>
       </c>
     </row>
@@ -899,16 +891,13 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="19" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
           <t>4.    OPERATING  CONDITIONS</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="B29" s="13" t="inlineStr">
@@ -954,6 +943,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="14" customHeight="1">
       <c r="B32" s="12" t="inlineStr">
         <is>
@@ -961,16 +951,13 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="19" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
         <is>
           <t>5.    SAFETY  INSULATION</t>
         </is>
       </c>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
     </row>
     <row r="35" ht="14" customHeight="1">
       <c r="B35" s="12" t="inlineStr">
@@ -1195,6 +1182,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="14" customHeight="1">
       <c r="B45" s="12" t="inlineStr">
         <is>

</xml_diff>